<commit_message>
Checkpoint before restoring Undo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-uploads/sample_departments.xlsx
+++ b/sample-uploads/sample_departments.xlsx
@@ -397,12 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
-  <cols>
-    <col min="1" max="1" width="44.83203125" customWidth="1"/>
-    <col min="2" max="2" width="8.83203125" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:D8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -414,6 +409,9 @@
       <c r="C1" t="str">
         <v>Dean</v>
       </c>
+      <c r="D1" t="str">
+        <v>Dean Email</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -425,6 +423,9 @@
       <c r="C2" t="str">
         <v>Dr. Maria Elena Santos</v>
       </c>
+      <c r="D2" t="str">
+        <v>mariaelena.santos@unc.edu.ph</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -436,6 +437,9 @@
       <c r="C3" t="str">
         <v>Dr. Teresita L. Gomez</v>
       </c>
+      <c r="D3" t="str">
+        <v>teresita.gomez@unc.edu.ph</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -445,7 +449,10 @@
         <v>SCIS</v>
       </c>
       <c r="C4" t="str">
-        <v>Dr. Evelyn S. Marquez</v>
+        <v>Edrian Lait</v>
+      </c>
+      <c r="D4" t="str">
+        <v>edrian.lait@unc.edu.ph</v>
       </c>
     </row>
     <row r="5">
@@ -458,6 +465,9 @@
       <c r="C5" t="str">
         <v>Atty. Ramon D. Fernandez</v>
       </c>
+      <c r="D5" t="str">
+        <v>ramon.fernandez@unc.edu.ph</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -469,6 +479,9 @@
       <c r="C6" t="str">
         <v>Dr. Carmela V. Reyes</v>
       </c>
+      <c r="D6" t="str">
+        <v>carmela.reyes@unc.edu.ph</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -480,6 +493,9 @@
       <c r="C7" t="str">
         <v>Engr. Ramon T. Villanueva</v>
       </c>
+      <c r="D7" t="str">
+        <v>ramon.villanueva@unc.edu.ph</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -491,10 +507,13 @@
       <c r="C8" t="str">
         <v>Dr. Lourdes A. Bautista</v>
       </c>
+      <c r="D8" t="str">
+        <v>lourdes.bautista@unc.edu.ph</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>